<commit_message>
chore: honest tracker update — 1 Done, 27 In Progress, 22 Todo (#1485)
Co-authored-by: Gurpreet <lifeofgurpreet@users.noreply.github.com>
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/archive/reports/deep-research/mereka_lms_top50_tracker.xlsx
+++ b/docs/archive/reports/deep-research/mereka_lms_top50_tracker.xlsx
@@ -566,12 +566,12 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo.html | https://docs.tutor.edly.io/install.html</t>
+          <t>Tutor 21 (Ulmo) is the baseline. Image builds working. But custom Dockerfile was dead code — only Tutor-generated Dockerfile matters. Node 18 needed for learner-record (webpack 4).</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/dev_op_release_notes.html</t>
+          <t>No Ulmo upgrade gap analysis done. Running Ulmo but haven't audited what changed.</t>
         </is>
       </c>
     </row>
@@ -676,12 +676,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/ulmo/community/release_notes/ulmo/design_tokens.html</t>
+          <t>Design tokens partially working. Mereka theme compiles. But branding per-tenant is NOT working — SOF/BB show Mereka pink (#1383).</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/olive/mfe_runtime_configuration.html</t>
+          <t>MFE config API serves 12+ keys per tenant. SiteConfiguration cleanup automated. BUT: SiteConfig overrides accumulate stale data. ConfigMap hash wiring (#1478) prevents seamless deploy.</t>
         </is>
       </c>
     </row>
@@ -786,12 +786,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/developers/concepts/hooks_extension_framework.html | https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0050-hooks-extension-framework.html</t>
+          <t>Tutor plugin architecture used. Custom apps in modules. BUT: 7 inline middleware copies across 3 overlays. Module imports from ConfigMap unreliable.</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0030-arch-pii-markup-and-auditing.html</t>
+          <t>No PII audit done.</t>
         </is>
       </c>
     </row>
@@ -896,12 +896,12 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/maple.html</t>
+          <t>Learning MFE deployed. BUT: learner dashboard shows 403 'bff.has_read_access' error on dev. Profile page blank. NOT actually working for real users.</t>
         </is>
       </c>
     </row>
@@ -951,12 +951,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>https://docs.tutor.edly.io/install.html</t>
+          <t>3 envs on RKE2 with ArgoCD. BUT: ConfigMap changes need hard refresh. Pod egress broken (#1460). Staging permanently Degraded (Ralph). NOT one-command reproducible.</t>
         </is>
       </c>
     </row>
@@ -1002,10 +1002,14 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>mysql-backup runs daily. auth-verify + cert-verify passing. BUT: restore drill NEVER done. ORA2/media on emptyDir. course-reindex blocked by networking.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1053,10 +1057,14 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Kyverno non-root + image signing policies. BUT: cosign GHCR auth fails for verification. No SBOM.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1104,12 +1112,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/ulmo/community/release_notes/ulmo/ulmo_rp.html</t>
+          <t>Admin Console MFE serves HTTP 200 with root div. BUT: not verified with real user — may have same issues as learner dashboard.</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1172,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/ulmo_rp.html</t>
+          <t>Content Libraries v2 not migrated. Legacy libraries only.</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1227,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/learners/sfd_notifications/index.html</t>
+          <t>Notifications not enabled.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1282,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/feature_release_notes.html</t>
+          <t>Catalog revamp not done.</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1337,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/feature_release_notes.html</t>
+          <t>LTI not configured.</t>
         </is>
       </c>
     </row>
@@ -1379,10 +1387,14 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>OIDC SSO via Authentik works for primary tenant. Studio SSO fixed. BUT: Enterprise SSO feature-flagged off. Multi-tenant OAuth chain works but Studio moment.js crash (#1385).</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1430,12 +1442,12 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/site_ops/aspects/index.html</t>
+          <t>Aspects ClickHouse + Superset on dev/staging. Prod dormant. Tracking logs ephemeral. ERB needs verification.</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1502,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/developers/concepts/hooks_extension_framework.html</t>
+          <t>No product metrics layer.</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1552,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/overhangio/tutor-discovery</t>
+          <t>Discovery service deployed. Health endpoint responds. BUT: discovery-sync CronJob status unverified after recent changes.</t>
         </is>
       </c>
     </row>
@@ -1595,12 +1607,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/overhangio/tutor-credentials | https://docs.openedx.org/en/latest/community/release_notes/teak/feature_release_notes.html</t>
+          <t>Credentials deployed. Learner Record MFE builds and serves on prod. BUT: dev learner-record 404 (image tag stale). Actual learner record functionality unverified.</t>
         </is>
       </c>
     </row>
@@ -1650,12 +1662,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/site_ops/install_configure_run_guide/ecommerce-deprecated/index.html | https://docs.openedx.org/en/latest/community/release_notes/quince/woocommerce.html</t>
+          <t>Oscar deprecated. Purchase Gateway spec exists. BUT: no actual commerce working.</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1717,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>https://openedx.org/blog/open-edx-sumac-release-is-here/</t>
+          <t>Meilisearch deployed and healthy. Forum uses it. BUT: Django SEARCH_ENGINE still says ElasticSearchEngine. course-reindex can't reach MongoDB. Search not actually verified from user perspective.</t>
         </is>
       </c>
     </row>
@@ -1760,12 +1772,12 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>https://openedx.org/blog/open-edx-sumac-release-is-here/ | https://docs.openedx.org/en/latest/community/release_notes/ulmo/ulmo_marketing_notes.html</t>
+          <t>Python openedx-forum in LMS. Discussions MFE serves. ENABLE_DISCUSSIONS_MFE set. BUT: not verified that forum content actually displays.</t>
         </is>
       </c>
     </row>
@@ -1815,10 +1827,14 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Prometheus + Grafana + Tempo + Loki on dev. ServiceMonitors deployed. BUT: alerting not proven end-to-end. No PagerDuty/Slack integration verified.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="80" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1871,7 +1887,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/eduNEXT/tutor-contrib-mfe-extensions</t>
+          <t>No CDN configured. No caching strategy beyond Caddy defaults.</t>
         </is>
       </c>
     </row>
@@ -1917,10 +1933,14 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Secure cookies with per-tenant domain scoping. JWT auth. Session middleware. BUT: SiteConfiguration stale overrides can break cookie domains.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="80" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -1968,12 +1988,12 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0048-brand-customization.html</t>
+          <t>3 tenants operational. Tenant-aware LMS redirect works. Studio OAuth tenant-aware. BUT: tenant homepages NOT branded per-tenant (#1383). Profile page broken. Learner dashboard BFF 403.</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2048,7 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0065-arch-frontend-composability.html</t>
+          <t>No OEP-65 module architecture adoption.</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2101,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>No WCAG audit done.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="80" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -2134,7 +2158,7 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/ulmo/community/release_notes/ulmo/design_tokens.html</t>
+          <t>Mobile readiness not verified.</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2209,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/developers/concepts/oep58.html | https://docs.openedx.org/en/open-release-sumac.master/developers/how-tos/maintain-translations-in-your-repo.html</t>
+          <t>Translation workflow not adopted.</t>
         </is>
       </c>
     </row>
@@ -2235,12 +2259,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/developers/concepts/hooks_extension_framework.html</t>
+          <t>Tutor plugin + patches. BUT: 7 inline middleware copies across overlays. Dead Dockerfile confusion. apply-patches.sh is monkey-patching.</t>
         </is>
       </c>
     </row>
@@ -2286,10 +2310,14 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>ruff + shellcheck + eslint configured. 162 CI scripts. BUT: CI release-gate flakes. Footer parity script was checking wrong section names until today.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="80" customHeight="1">
       <c r="A35" s="2" t="n">
@@ -2337,10 +2365,14 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>162 static scripts. Fixture replay. Smoke accounts. BUT: NO real Playwright E2E. All 'proof' was curl HTTP 200 which misses JS errors, 403s, blank pages.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="80" customHeight="1">
       <c r="A36" s="2" t="n">
@@ -2391,7 +2423,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>No API documentation.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="80" customHeight="1">
       <c r="A37" s="2" t="n">
@@ -2439,10 +2475,14 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Troubleshooting runbook exists. CI/CD docs exist. BUT: restore drill runbook not created. Operational procedures incomplete.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="80" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -2490,12 +2530,12 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0048-brand-customization.html</t>
+          <t>Brand package (@edx/brand) in MFE builds. Footer data in API. BUT: per-tenant branding NOT working. SOF/BB show Mereka colors.</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2584,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Repo not restructured. Still flat scripts/ with 162+ files.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="80" customHeight="1">
       <c r="A40" s="2" t="n">
@@ -2595,7 +2639,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>No golden path dev environment.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="80" customHeight="1">
       <c r="A41" s="2" t="n">
@@ -2646,7 +2694,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>No semantic versioning. No release process.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="80" customHeight="1">
       <c r="A42" s="2" t="n">
@@ -2694,10 +2746,14 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>RKE2 + ArgoCD + Kustomize. bbi-infrastructure repo. BUT: ConfigMap wiring broken (#1478). Vendor sync manual (#1387). Pod egress broken (#1460).</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="80" customHeight="1">
       <c r="A43" s="2" t="n">
@@ -2745,10 +2801,14 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Infisical → ESO → K8s Secrets pipeline works. Machine identity auth. Pre-commit secret scanning.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="80" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -2797,7 +2857,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/processes/oep-0021-proc-deprecation.html</t>
+          <t>No deprecation discipline adopted.</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2912,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0030-arch-pii-markup-and-auditing.html</t>
+          <t>No data retention policy.</t>
         </is>
       </c>
     </row>
@@ -2902,12 +2962,12 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/feature_release_notes.html | https://docs.openedx.org/projects/openedx-proposals/en/latest/architectural-decisions/oep-0065-arch-frontend-composability.html</t>
+          <t>Plugin slots partially used. Footer component. BUT: MFE slot ownership stripped by patch. Not fully migrated to plugin slots.</t>
         </is>
       </c>
     </row>
@@ -2957,10 +3017,14 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K47" s="3" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>ARC runners build images. GHCR push works. Release object + truth ledger emit. BUT: dispatch blocked by GitHub App permissions. Manual promotion only.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="80" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -3013,7 +3077,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/ulmo/feature_release_notes.html</t>
+          <t>No admin tooling consolidation.</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3130,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K49" s="3" t="inlineStr"/>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>No capacity planning.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="80" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -3117,7 +3185,11 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="K50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>No audit logging.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="80" customHeight="1">
       <c r="A51" s="2" t="n">
@@ -3170,7 +3242,7 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>https://docs.openedx.org/en/latest/community/release_notes/index.html</t>
+          <t>No upgrade-every-release discipline.</t>
         </is>
       </c>
     </row>

</xml_diff>